<commit_message>
update terbaru paling baru
</commit_message>
<xml_diff>
--- a/public/Database_Template.xlsx
+++ b/public/Database_Template.xlsx
@@ -397,7 +397,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W2"/>
+  <dimension ref="A1:X2"/>
+  <cols>
+    <col min="24" max="24" width="22" hidden="0" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -468,6 +471,9 @@
       </c>
       <c r="W1" t="str">
         <v xml:space="preserve">Company Website </v>
+      </c>
+      <c r="X1" t="str">
+        <v>Cabang/Kantor</v>
       </c>
     </row>
     <row r="2">

</xml_diff>

<commit_message>
Upgrade Next.js and add CRM dashboard charts and EMS v2
Use patched Next16 and React19, refresh CRM analytics views, and support per-event legacy/v2 EMS selection. Keep EO Scout and TAGTOG changes out of this commit.
</commit_message>
<xml_diff>
--- a/public/Database_Template.xlsx
+++ b/public/Database_Template.xlsx
@@ -64,8 +64,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -399,155 +402,158 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:X2"/>
   <cols>
-    <col min="21" max="21" width="22" hidden="0" customWidth="1"/>
+    <col min="1" max="20" style="1" width="9.140625" hidden="0" customWidth="1"/>
+    <col min="21" max="21" width="22" hidden="0" customWidth="1" style="1"/>
+    <col min="22" max="24" style="1" width="9.140625" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
+      <c r="A1" t="str" s="0">
         <v>No</v>
       </c>
-      <c r="B1" t="str">
+      <c r="B1" t="str" s="0">
         <v>Nama Group/Holding Company</v>
       </c>
-      <c r="C1" t="str">
+      <c r="C1" t="str" s="0">
         <v>Nama Brand</v>
       </c>
-      <c r="D1" t="str">
+      <c r="D1" t="str" s="0">
         <v>Company Name</v>
       </c>
-      <c r="E1" t="str">
+      <c r="E1" t="str" s="0">
         <v>Salutation</v>
       </c>
-      <c r="F1" t="str">
+      <c r="F1" t="str" s="0">
         <v>First Name</v>
       </c>
-      <c r="G1" t="str">
+      <c r="G1" t="str" s="0">
         <v>Last Name</v>
       </c>
-      <c r="H1" t="str">
+      <c r="H1" t="str" s="0">
         <v>Position</v>
       </c>
-      <c r="I1" t="str">
+      <c r="I1" t="str" s="0">
         <v>Division</v>
       </c>
-      <c r="J1" t="str">
+      <c r="J1" t="str" s="0">
         <v>Jobtitle</v>
       </c>
-      <c r="K1" t="str">
+      <c r="K1" t="str" s="0">
         <v>Address</v>
       </c>
-      <c r="L1" t="str">
+      <c r="L1" t="str" s="0">
         <v>Office Phone</v>
       </c>
-      <c r="M1" t="str">
+      <c r="M1" t="str" s="0">
         <v>Mobile Phone</v>
       </c>
-      <c r="N1" t="str">
+      <c r="N1" t="str" s="0">
         <v>Company Email Address</v>
       </c>
-      <c r="O1" t="str">
+      <c r="O1" t="str" s="0">
         <v xml:space="preserve"> Personal Email Address</v>
       </c>
-      <c r="P1" t="str">
+      <c r="P1" t="str" s="0">
         <v>Industry</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="Q1" t="str" s="0">
         <v>Company Size (Revenue)</v>
       </c>
-      <c r="R1" t="str">
+      <c r="R1" t="str" s="0">
         <v>Company Size (Employee)</v>
       </c>
-      <c r="S1" t="str">
+      <c r="S1" t="str" s="0">
         <v>Company Hardware</v>
       </c>
-      <c r="T1" t="str">
+      <c r="T1" t="str" s="0">
         <v>Linkedin Link</v>
       </c>
-      <c r="U1" t="str">
+      <c r="U1" t="str" s="0">
         <v>Cabang/Kantor</v>
       </c>
-      <c r="V1" t="str">
+      <c r="V1" t="str" s="0">
         <v>City</v>
       </c>
-      <c r="W1" t="str">
+      <c r="W1" t="str" s="0">
         <v>Postal Code</v>
       </c>
-      <c r="X1" t="str">
+      <c r="X1" t="str" s="0">
         <v xml:space="preserve">Company Website </v>
       </c>
     </row>
     <row r="2">
-      <c r="A2">
+      <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" t="str">
+      <c r="B2" t="str" s="1">
         <v>Astra Group</v>
       </c>
-      <c r="C2" t="str">
+      <c r="C2" t="str" s="1">
         <v>Daihatsu</v>
       </c>
-      <c r="D2" t="str">
+      <c r="D2" t="str" s="1">
         <v xml:space="preserve"> Astra Daihatsu Motor PT</v>
       </c>
-      <c r="E2" t="str">
+      <c r="E2" t="str" s="1">
         <v>Ms</v>
       </c>
-      <c r="F2" t="str">
+      <c r="F2" t="str" s="1">
         <v>Jasmine</v>
       </c>
-      <c r="G2" t="str">
+      <c r="G2" t="str" s="1">
         <v xml:space="preserve"> Kezia</v>
       </c>
-      <c r="H2" t="str">
+      <c r="H2" t="str" s="1">
         <v>C-level//GM/Director</v>
       </c>
-      <c r="I2" t="str">
+      <c r="I2" t="str" s="1">
         <v>IT Infrastructure</v>
       </c>
-      <c r="J2" t="str">
+      <c r="J2" t="str" s="1">
         <v xml:space="preserve">Information Technology Supervisor </v>
       </c>
-      <c r="K2" t="str">
+      <c r="K2" t="str" s="1">
         <v>Jl. Gaya Motor III No. 5, Sunter II, Jakarta Utara 14330</v>
       </c>
-      <c r="L2" t="str">
+      <c r="L2" t="str" s="1">
         <v>(021) 6510300</v>
       </c>
-      <c r="M2">
+      <c r="M2" s="1">
         <v>6282124322804</v>
       </c>
-      <c r="N2" t="str">
+      <c r="N2" t="str" s="1">
         <v>jasminekezia14@astra.co.id</v>
       </c>
-      <c r="O2" t="str">
+      <c r="O2" t="str" s="1">
         <v>hisyamagung20@gmail.com</v>
       </c>
-      <c r="P2" t="str">
+      <c r="P2" t="str" s="1">
         <v>telecommunications</v>
       </c>
-      <c r="Q2" t="str">
+      <c r="Q2" t="str" s="1">
         <v/>
       </c>
-      <c r="R2" t="str">
+      <c r="R2" t="str" s="1">
         <v>100-1000</v>
       </c>
-      <c r="S2" t="str">
+      <c r="S2" t="str" s="1">
         <v/>
       </c>
-      <c r="T2" t="str">
+      <c r="T2" t="str" s="1">
         <v>https://www.linkedin.com/in/jasmine-kezia-476208165/</v>
       </c>
-      <c r="V2" t="str">
+      <c r="V2" t="str" s="1">
         <v>Jakarta</v>
       </c>
-      <c r="W2" t="str">
+      <c r="W2" t="str" s="1">
         <v/>
       </c>
-      <c r="X2" t="str">
+      <c r="X2" t="str" s="1">
         <v>http://daihatsu.co.id/</v>
       </c>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1" formatCells="1" formatColumns="0" formatRows="0" insertColumns="1" insertRows="1" deleteColumns="1" deleteRows="1" selectLockedCells="0" selectUnlockedCells="0"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:T2 V1:X2"/>
   </ignoredErrors>

</xml_diff>